<commit_message>
feat(MK): update for modding integration 3
</commit_message>
<xml_diff>
--- a/ModdingKit/package/LangMod/EN/EScriptLang.xlsx
+++ b/ModdingKit/package/LangMod/EN/EScriptLang.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\Elin.Plugins\ModdingKit\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5920EC9-64BC-4D80-9E5F-4FB95C13D9A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFA6935-EF5F-4693-95A1-57A12FD6B165}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="225" yWindow="1620" windowWidth="25965" windowHeight="15615" tabRatio="555" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23070" yWindow="3555" windowWidth="25965" windowHeight="15615" tabRatio="555" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="71">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -515,13 +515,33 @@
   </si>
   <si>
     <t>es_ui_invalid_patch</t>
+  </si>
+  <si>
+    <t>enableModError</t>
+  </si>
+  <si>
+    <t>Enable Error Popup</t>
+  </si>
+  <si>
+    <t>errorPopup_tip</t>
+  </si>
+  <si>
+    <t>When enabled, in-game errors will be shown in a popup along with any mods that may be causing them.
+Useful for debugging mod‑related problems and sending reports to mod creators.</t>
+  </si>
+  <si>
+    <t>有効にすると、ゲームプレイ中に発生したエラーをポップアップで表示し、原因の可能性があるMODをあわせて表示します。
+MOD関連の問題のデバッグや、MOD作者への報告に役立ちます。</t>
+  </si>
+  <si>
+    <t>エラー表示を有効にする</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -580,13 +600,6 @@
     <font>
       <sz val="15.8"/>
       <color theme="1"/>
-      <name val="Cascadia Code"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
-    <font>
-      <sz val="15.8"/>
-      <color theme="1"/>
       <name val="Yu Gothic"/>
       <family val="3"/>
       <charset val="128"/>
@@ -612,7 +625,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -635,9 +648,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1170,10 +1180,10 @@
         <v>58</v>
       </c>
       <c r="B21" s="4"/>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="5" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1182,10 +1192,10 @@
         <v>64</v>
       </c>
       <c r="B22" s="4"/>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="5" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1202,28 +1212,40 @@
       </c>
     </row>
     <row r="24" spans="1:4" ht="23.25">
-      <c r="A24" s="6"/>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-    </row>
-    <row r="25" spans="1:4" ht="23.25">
-      <c r="A25" s="6"/>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
+      <c r="A24" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" s="4"/>
+      <c r="C24" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="69.75">
+      <c r="A25" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B25" s="4"/>
+      <c r="C25" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="26" spans="1:4" ht="23.25">
-      <c r="A26" s="6"/>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
     </row>
     <row r="27" spans="1:4" ht="23.25">
-      <c r="A27" s="6"/>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
feat(MK): add default scripting namespaces
</commit_message>
<xml_diff>
--- a/ModdingKit/package/LangMod/EN/EScriptLang.xlsx
+++ b/ModdingKit/package/LangMod/EN/EScriptLang.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\Elin.Plugins\ModdingKit\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFA6935-EF5F-4693-95A1-57A12FD6B165}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ADCCAE0-6FD2-4F7A-97C8-1507DB316674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23070" yWindow="3555" windowWidth="25965" windowHeight="15615" tabRatio="555" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18780" yWindow="1485" windowWidth="31695" windowHeight="18195" tabRatio="555" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -481,6 +481,36 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>es_warn_missing_method</t>
+  </si>
+  <si>
+    <t>es_ui_invalid_patch</t>
+  </si>
+  <si>
+    <t>enableModError</t>
+  </si>
+  <si>
+    <t>Enable Error Popup</t>
+  </si>
+  <si>
+    <t>errorPopup_tip</t>
+  </si>
+  <si>
+    <t>When enabled, in-game errors will be shown in a popup along with any mods that may be causing them.
+Useful for debugging mod‑related problems and sending reports to mod creators.</t>
+  </si>
+  <si>
+    <t>有効にすると、ゲームプレイ中に発生したエラーをポップアップで表示し、原因の可能性があるMODをあわせて表示します。
+MOD関連の問題のデバッグや、MOD作者への報告に役立ちます。</t>
+  </si>
+  <si>
+    <t>エラー表示を有効にする</t>
+  </si>
+  <si>
+    <t>&lt;color=#d343f7&gt;A mod is incompatible with your game version.&lt;/color&gt;
+#1</t>
+  </si>
+  <si>
     <r>
       <t>&lt;color=#d343f7&gt;MOD</t>
     </r>
@@ -502,39 +532,8 @@
         <family val="3"/>
       </rPr>
       <t>&lt;/color&gt;
-{0}</t>
-    </r>
-  </si>
-  <si>
-    <t>&lt;color=#d343f7&gt;A mod is incompatible with your game version.&lt;/color&gt;
-{0}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>es_warn_missing_method</t>
-  </si>
-  <si>
-    <t>es_ui_invalid_patch</t>
-  </si>
-  <si>
-    <t>enableModError</t>
-  </si>
-  <si>
-    <t>Enable Error Popup</t>
-  </si>
-  <si>
-    <t>errorPopup_tip</t>
-  </si>
-  <si>
-    <t>When enabled, in-game errors will be shown in a popup along with any mods that may be causing them.
-Useful for debugging mod‑related problems and sending reports to mod creators.</t>
-  </si>
-  <si>
-    <t>有効にすると、ゲームプレイ中に発生したエラーをポップアップで表示し、原因の可能性があるMODをあわせて表示します。
-MOD関連の問題のデバッグや、MOD作者への報告に役立ちます。</t>
-  </si>
-  <si>
-    <t>エラー表示を有効にする</t>
+#1</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1189,7 +1188,7 @@
     </row>
     <row r="22" spans="1:4" ht="25.5">
       <c r="A22" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="5" t="s">
@@ -1201,38 +1200,38 @@
     </row>
     <row r="23" spans="1:4" ht="48.75">
       <c r="A23" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="5" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="23.25">
       <c r="A24" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="69.75">
       <c r="A25" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="23.25">

</xml_diff>